<commit_message>
Prepare backend for production
</commit_message>
<xml_diff>
--- a/storage/registrations/IEEE-GU-Event-Registrations.xlsx
+++ b/storage/registrations/IEEE-GU-Event-Registrations.xlsx
@@ -7,13 +7,16 @@
     <sheet sheetId="1" name="IEEE GU Technical Workshop" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="new event" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="event test" state="visible" r:id="rId6"/>
+    <sheet sheetId="5" name="single event test new" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="test event team" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="team test 2" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="94">
   <si>
     <t>Registration ID</t>
   </si>
@@ -133,6 +136,168 @@
   </si>
   <si>
     <t>cmu5b7adz0008dsv6sxaj6tyk</t>
+  </si>
+  <si>
+    <t>Team Name</t>
+  </si>
+  <si>
+    <t>Team Leader</t>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Email Address</t>
+  </si>
+  <si>
+    <t>Mobile Number</t>
+  </si>
+  <si>
+    <t>Department (2)</t>
+  </si>
+  <si>
+    <t>Course (2)</t>
+  </si>
+  <si>
+    <t>Academic Year</t>
+  </si>
+  <si>
+    <t>Roll Number (2)</t>
+  </si>
+  <si>
+    <t>IEEE Membership Number (2)</t>
+  </si>
+  <si>
+    <t>cmu9una9n00003cv6zrgtxlr9</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>cmu9wcvke00028wv64pv1i5vm</t>
+  </si>
+  <si>
+    <t>himeshroy.cse@gmail.com</t>
+  </si>
+  <si>
+    <t>102638195</t>
+  </si>
+  <si>
+    <t>CSE</t>
+  </si>
+  <si>
+    <t>B.Tech CSE AI ML</t>
+  </si>
+  <si>
+    <t>2nd</t>
+  </si>
+  <si>
+    <t>Team Name (2)</t>
+  </si>
+  <si>
+    <t>cmu9nmyg80011j0v6ha0c08n0</t>
+  </si>
+  <si>
+    <t>XZY</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>cmua08llj0001z8v6tzxoyl1p</t>
+  </si>
+  <si>
+    <t>royhimqws36@gmail.com</t>
+  </si>
+  <si>
+    <t>sad</t>
+  </si>
+  <si>
+    <t>sshudwjjjjjjjjjj</t>
+  </si>
+  <si>
+    <t>65926131655</t>
+  </si>
+  <si>
+    <t>frf</t>
+  </si>
+  <si>
+    <t>ewaksdlad</t>
+  </si>
+  <si>
+    <t>cmua08m08000bz8v6n7pr6cj6</t>
+  </si>
+  <si>
+    <t>royhimqws36hh@gmail.com</t>
+  </si>
+  <si>
+    <t>cmua0su4d000mz8v6u9y7bqj8</t>
+  </si>
+  <si>
+    <t>fdfdgg</t>
+  </si>
+  <si>
+    <t>royhim23fffffff6@gmail.com</t>
+  </si>
+  <si>
+    <t>dsddd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fdfdgg </t>
+  </si>
+  <si>
+    <t>cmua0suh7000wz8v6ay7kahlr</t>
+  </si>
+  <si>
+    <t>dddddddddd</t>
+  </si>
+  <si>
+    <t>royhimes55qq4@gmail.com</t>
+  </si>
+  <si>
+    <t>0000000000</t>
+  </si>
+  <si>
+    <t>ghvhgv</t>
+  </si>
+  <si>
+    <t>hjbhhhhhhhhhhh</t>
+  </si>
+  <si>
+    <t>871178777777778</t>
+  </si>
+  <si>
+    <t>iiiiiiiii</t>
+  </si>
+  <si>
+    <t>cmua1dvoy0017z8v6w0uxjcv8</t>
+  </si>
+  <si>
+    <t>XZYYYYYYg</t>
+  </si>
+  <si>
+    <t>abcaedj@gmail.com</t>
+  </si>
+  <si>
+    <t>sjzdf</t>
+  </si>
+  <si>
+    <t>9655582255</t>
+  </si>
+  <si>
+    <t>akakak</t>
+  </si>
+  <si>
+    <t>cmua1dw0y001gz8v6mcgsqfcw</t>
+  </si>
+  <si>
+    <t>abcaedjg@gmail.com</t>
+  </si>
+  <si>
+    <t>cmua1dwc5001oz8v6kypwybg5</t>
+  </si>
+  <si>
+    <t>abcaedjhjj@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -317,6 +482,172 @@
     <tableColumn id="11" name="Registration Status" totalsRowFunction="none"/>
     <tableColumn id="12" name="Registered At" totalsRowFunction="none"/>
     <tableColumn id="13" name="Attended At" totalsRowFunction="none"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" name="Event_single_event_test_new_cmu9n2619000jj0v6a4wcfdbs" displayName="Event_single_event_test_new_cmu9n2619000jj0v6a4wcfdbs" ref="A1:W1" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:W1">
+    <filterColumn colId="0" hiddenButton="0"/>
+    <filterColumn colId="1" hiddenButton="0"/>
+    <filterColumn colId="2" hiddenButton="0"/>
+    <filterColumn colId="3" hiddenButton="0"/>
+    <filterColumn colId="4" hiddenButton="0"/>
+    <filterColumn colId="5" hiddenButton="0"/>
+    <filterColumn colId="6" hiddenButton="0"/>
+    <filterColumn colId="7" hiddenButton="0"/>
+    <filterColumn colId="8" hiddenButton="0"/>
+    <filterColumn colId="9" hiddenButton="0"/>
+    <filterColumn colId="10" hiddenButton="0"/>
+    <filterColumn colId="11" hiddenButton="0"/>
+    <filterColumn colId="12" hiddenButton="0"/>
+    <filterColumn colId="13" hiddenButton="0"/>
+    <filterColumn colId="14" hiddenButton="0"/>
+    <filterColumn colId="15" hiddenButton="0"/>
+    <filterColumn colId="16" hiddenButton="0"/>
+    <filterColumn colId="17" hiddenButton="0"/>
+    <filterColumn colId="18" hiddenButton="0"/>
+    <filterColumn colId="19" hiddenButton="0"/>
+    <filterColumn colId="20" hiddenButton="0"/>
+    <filterColumn colId="21" hiddenButton="0"/>
+    <filterColumn colId="22" hiddenButton="0"/>
+  </autoFilter>
+  <tableColumns count="23">
+    <tableColumn id="1" name="Registration ID" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="Name" totalsRowFunction="none"/>
+    <tableColumn id="3" name="Email" totalsRowFunction="none"/>
+    <tableColumn id="4" name="Phone" totalsRowFunction="none"/>
+    <tableColumn id="5" name="IEEE Membership Number" totalsRowFunction="none"/>
+    <tableColumn id="6" name="Membership Status" totalsRowFunction="none"/>
+    <tableColumn id="7" name="Department" totalsRowFunction="none"/>
+    <tableColumn id="8" name="Course" totalsRowFunction="none"/>
+    <tableColumn id="9" name="Year" totalsRowFunction="none"/>
+    <tableColumn id="10" name="Roll Number" totalsRowFunction="none"/>
+    <tableColumn id="11" name="Team Name" totalsRowFunction="none"/>
+    <tableColumn id="12" name="Team Leader" totalsRowFunction="none"/>
+    <tableColumn id="13" name="Registration Status" totalsRowFunction="none"/>
+    <tableColumn id="14" name="Registered At" totalsRowFunction="none"/>
+    <tableColumn id="15" name="Attended At" totalsRowFunction="none"/>
+    <tableColumn id="16" name="Full Name" totalsRowFunction="none"/>
+    <tableColumn id="17" name="Email Address" totalsRowFunction="none"/>
+    <tableColumn id="18" name="Mobile Number" totalsRowFunction="none"/>
+    <tableColumn id="19" name="Department (2)" totalsRowFunction="none"/>
+    <tableColumn id="20" name="Course (2)" totalsRowFunction="none"/>
+    <tableColumn id="21" name="Academic Year" totalsRowFunction="none"/>
+    <tableColumn id="22" name="Roll Number (2)" totalsRowFunction="none"/>
+    <tableColumn id="23" name="IEEE Membership Number (2)" totalsRowFunction="none"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" name="Event_test_event_team_cmu9g023h0002vov6pcitlc0f" displayName="Event_test_event_team_cmu9g023h0002vov6pcitlc0f" ref="A1:W1" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:W1">
+    <filterColumn colId="0" hiddenButton="0"/>
+    <filterColumn colId="1" hiddenButton="0"/>
+    <filterColumn colId="2" hiddenButton="0"/>
+    <filterColumn colId="3" hiddenButton="0"/>
+    <filterColumn colId="4" hiddenButton="0"/>
+    <filterColumn colId="5" hiddenButton="0"/>
+    <filterColumn colId="6" hiddenButton="0"/>
+    <filterColumn colId="7" hiddenButton="0"/>
+    <filterColumn colId="8" hiddenButton="0"/>
+    <filterColumn colId="9" hiddenButton="0"/>
+    <filterColumn colId="10" hiddenButton="0"/>
+    <filterColumn colId="11" hiddenButton="0"/>
+    <filterColumn colId="12" hiddenButton="0"/>
+    <filterColumn colId="13" hiddenButton="0"/>
+    <filterColumn colId="14" hiddenButton="0"/>
+    <filterColumn colId="15" hiddenButton="0"/>
+    <filterColumn colId="16" hiddenButton="0"/>
+    <filterColumn colId="17" hiddenButton="0"/>
+    <filterColumn colId="18" hiddenButton="0"/>
+    <filterColumn colId="19" hiddenButton="0"/>
+    <filterColumn colId="20" hiddenButton="0"/>
+    <filterColumn colId="21" hiddenButton="0"/>
+    <filterColumn colId="22" hiddenButton="0"/>
+  </autoFilter>
+  <tableColumns count="23">
+    <tableColumn id="1" name="Registration ID" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="Name" totalsRowFunction="none"/>
+    <tableColumn id="3" name="Email" totalsRowFunction="none"/>
+    <tableColumn id="4" name="Phone" totalsRowFunction="none"/>
+    <tableColumn id="5" name="IEEE Membership Number" totalsRowFunction="none"/>
+    <tableColumn id="6" name="Membership Status" totalsRowFunction="none"/>
+    <tableColumn id="7" name="Department" totalsRowFunction="none"/>
+    <tableColumn id="8" name="Course" totalsRowFunction="none"/>
+    <tableColumn id="9" name="Year" totalsRowFunction="none"/>
+    <tableColumn id="10" name="Roll Number" totalsRowFunction="none"/>
+    <tableColumn id="11" name="Team Name" totalsRowFunction="none"/>
+    <tableColumn id="12" name="Team Leader" totalsRowFunction="none"/>
+    <tableColumn id="13" name="Registration Status" totalsRowFunction="none"/>
+    <tableColumn id="14" name="Registered At" totalsRowFunction="none"/>
+    <tableColumn id="15" name="Attended At" totalsRowFunction="none"/>
+    <tableColumn id="16" name="Team Name (2)" totalsRowFunction="none"/>
+    <tableColumn id="17" name="Full Name" totalsRowFunction="none"/>
+    <tableColumn id="18" name="Email Address" totalsRowFunction="none"/>
+    <tableColumn id="19" name="Mobile Number" totalsRowFunction="none"/>
+    <tableColumn id="20" name="Department (2)" totalsRowFunction="none"/>
+    <tableColumn id="21" name="Course (2)" totalsRowFunction="none"/>
+    <tableColumn id="22" name="Academic Year" totalsRowFunction="none"/>
+    <tableColumn id="23" name="Roll Number (2)" totalsRowFunction="none"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" name="Event_team_test_2_cmu9qaebt0000i8v621k7kboi" displayName="Event_team_test_2_cmu9qaebt0000i8v621k7kboi" ref="A1:V1" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:V1">
+    <filterColumn colId="0" hiddenButton="0"/>
+    <filterColumn colId="1" hiddenButton="0"/>
+    <filterColumn colId="2" hiddenButton="0"/>
+    <filterColumn colId="3" hiddenButton="0"/>
+    <filterColumn colId="4" hiddenButton="0"/>
+    <filterColumn colId="5" hiddenButton="0"/>
+    <filterColumn colId="6" hiddenButton="0"/>
+    <filterColumn colId="7" hiddenButton="0"/>
+    <filterColumn colId="8" hiddenButton="0"/>
+    <filterColumn colId="9" hiddenButton="0"/>
+    <filterColumn colId="10" hiddenButton="0"/>
+    <filterColumn colId="11" hiddenButton="0"/>
+    <filterColumn colId="12" hiddenButton="0"/>
+    <filterColumn colId="13" hiddenButton="0"/>
+    <filterColumn colId="14" hiddenButton="0"/>
+    <filterColumn colId="15" hiddenButton="0"/>
+    <filterColumn colId="16" hiddenButton="0"/>
+    <filterColumn colId="17" hiddenButton="0"/>
+    <filterColumn colId="18" hiddenButton="0"/>
+    <filterColumn colId="19" hiddenButton="0"/>
+    <filterColumn colId="20" hiddenButton="0"/>
+    <filterColumn colId="21" hiddenButton="0"/>
+  </autoFilter>
+  <tableColumns count="22">
+    <tableColumn id="1" name="Registration ID" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="Name" totalsRowFunction="none"/>
+    <tableColumn id="3" name="Email" totalsRowFunction="none"/>
+    <tableColumn id="4" name="Phone" totalsRowFunction="none"/>
+    <tableColumn id="5" name="IEEE Membership Number" totalsRowFunction="none"/>
+    <tableColumn id="6" name="Membership Status" totalsRowFunction="none"/>
+    <tableColumn id="7" name="Department" totalsRowFunction="none"/>
+    <tableColumn id="8" name="Course" totalsRowFunction="none"/>
+    <tableColumn id="9" name="Year" totalsRowFunction="none"/>
+    <tableColumn id="10" name="Roll Number" totalsRowFunction="none"/>
+    <tableColumn id="11" name="Team Name" totalsRowFunction="none"/>
+    <tableColumn id="12" name="Team Leader" totalsRowFunction="none"/>
+    <tableColumn id="13" name="Registration Status" totalsRowFunction="none"/>
+    <tableColumn id="14" name="Registered At" totalsRowFunction="none"/>
+    <tableColumn id="15" name="Attended At" totalsRowFunction="none"/>
+    <tableColumn id="16" name="Team Name (2)" totalsRowFunction="none"/>
+    <tableColumn id="17" name="Full Name" totalsRowFunction="none"/>
+    <tableColumn id="18" name="Email Address" totalsRowFunction="none"/>
+    <tableColumn id="19" name="Mobile Number" totalsRowFunction="none"/>
+    <tableColumn id="20" name="Department (2)" totalsRowFunction="none"/>
+    <tableColumn id="21" name="Course (2)" totalsRowFunction="none"/>
+    <tableColumn id="22" name="Roll Number (2)" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1088,6 +1419,989 @@
   </sheetData>
   <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:W6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="24" customWidth="1"/>
+    <col min="4" max="5" width="24" style="1" customWidth="1"/>
+    <col min="6" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="24" style="1" customWidth="1"/>
+    <col min="11" max="13" width="24" customWidth="1"/>
+    <col min="14" max="15" width="24" style="2" customWidth="1"/>
+    <col min="16" max="23" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" s="8">
+        <v>46285.42335675926</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="8">
+        <v>46285.668323969905</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V3" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="W3" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="8">
+        <v>46285.668330092594</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="S4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="W4" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="8">
+        <v>46285.67925181713</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V5" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="W5" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="8">
+        <v>46285.67925716435</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V6" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="W6" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:W1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:W3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="24" customWidth="1"/>
+    <col min="4" max="5" width="24" style="1" customWidth="1"/>
+    <col min="6" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="24" style="1" customWidth="1"/>
+    <col min="11" max="13" width="24" customWidth="1"/>
+    <col min="14" max="15" width="24" style="2" customWidth="1"/>
+    <col min="16" max="23" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N2" s="8">
+        <v>46285.55961401621</v>
+      </c>
+      <c r="O2" s="8">
+        <v>46285.58092658565</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="8">
+        <v>46285.59287349537</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="V3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="W3" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:W1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:V4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="24" customWidth="1"/>
+    <col min="4" max="5" width="24" style="1" customWidth="1"/>
+    <col min="6" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="24" style="1" customWidth="1"/>
+    <col min="11" max="13" width="24" customWidth="1"/>
+    <col min="14" max="15" width="24" style="2" customWidth="1"/>
+    <col min="16" max="22" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" s="8">
+        <v>46285.690615405096</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="S2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="8">
+        <v>46285.69062039352</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V3" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="8">
+        <v>46285.69062505787</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="S4" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:V1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>